<commit_message>
melhoria readme + melhoria static
</commit_message>
<xml_diff>
--- a/data/2025-01-05_processos.xlsx
+++ b/data/2025-01-05_processos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -812,6 +812,38 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12345/2023</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>João da Silva</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>123.456.789-00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>['Empresa XYZ', 'Fulano de Tal']</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>['987.654.321-00', '111.222.333-44']</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>